<commit_message>
removing all historic data, adding in tab2 message to return to user input tab if no data uploaded yet
</commit_message>
<xml_diff>
--- a/www/scenario-template.xlsx
+++ b/www/scenario-template.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="86" documentId="13_ncr:1_{D4A44570-08E8-4318-9463-3D1D60012C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{364390A2-02A6-400B-8F6D-4339887006BD}"/>
   <bookViews>
-    <workbookView xWindow="2205" yWindow="1260" windowWidth="25875" windowHeight="18375" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="38700" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
changing user inpout tab data downlaod to handle the data validation in the worksheet that will maintain certain selection list inputs in the intervention type columns
</commit_message>
<xml_diff>
--- a/www/scenario-template.xlsx
+++ b/www/scenario-template.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pathseattle-my.sharepoint.com/personal/hthompson_path_org/Documents/Documents/github/malaria-budgeting-tool/www/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="86" documentId="13_ncr:1_{D4A44570-08E8-4318-9463-3D1D60012C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{364390A2-02A6-400B-8F6D-4339887006BD}"/>
+  <xr:revisionPtr revIDLastSave="87" documentId="13_ncr:1_{D4A44570-08E8-4318-9463-3D1D60012C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00C07003-1F6B-4ECC-8580-4857BE2B635C}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="38700" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="2205" windowWidth="38700" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="2025" sheetId="1" r:id="rId1"/>
+    <sheet name="template" sheetId="1" r:id="rId1"/>
     <sheet name="list-options-ignore" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>

</xml_diff>